<commit_message>
Checkpoint: Implementar limpieza masiva segura: 1. Endpoint wallet.dismissHistoricalReserveSuggestions: marca como 'dismissed' solo suggestions con status='suggested' createdAt < hoy 2. NO toca status='completed' ni wallet balance 3. Retorna countDismissed, reservedPendingBefore, reservedPendingAfter 4. Botón "Dismiss Historical Suggestions" en SuggestedTransfersCard con feedback visual 5. Test unitario para validar lógica de dismissal
</commit_message>
<xml_diff>
--- a/comparison.xlsx
+++ b/comparison.xlsx
@@ -430,13 +430,13 @@
         <v>Enero</v>
       </c>
       <c r="B4" t="str">
-        <v>3,921.754</v>
+        <v>3,155.89</v>
       </c>
       <c r="C4" t="str">
-        <v>$13,961.97</v>
+        <v>$14,921.71</v>
       </c>
       <c r="D4" t="str">
-        <v>$6,783.95</v>
+        <v>$5,009.56</v>
       </c>
     </row>
     <row r="5">
@@ -444,13 +444,13 @@
         <v>Febrero</v>
       </c>
       <c r="B5" t="str">
-        <v>3,835.398</v>
+        <v>3,613.509</v>
       </c>
       <c r="C5" t="str">
-        <v>$12,888.37</v>
+        <v>$14,837.88</v>
       </c>
       <c r="D5" t="str">
-        <v>$6,130.69</v>
+        <v>$5,531.33</v>
       </c>
     </row>
     <row r="6">
@@ -458,13 +458,13 @@
         <v>Marzo</v>
       </c>
       <c r="B6" t="str">
-        <v>3,881.993</v>
+        <v>3,061.74</v>
       </c>
       <c r="C6" t="str">
-        <v>$12,072.04</v>
+        <v>$12,195.96</v>
       </c>
       <c r="D6" t="str">
-        <v>$5,623.90</v>
+        <v>$6,262.18</v>
       </c>
     </row>
     <row r="7">
@@ -472,13 +472,13 @@
         <v>Abril</v>
       </c>
       <c r="B7" t="str">
-        <v>3,718.643</v>
+        <v>3,288.855</v>
       </c>
       <c r="C7" t="str">
-        <v>$12,332.17</v>
+        <v>$13,292.28</v>
       </c>
       <c r="D7" t="str">
-        <v>$5,613.19</v>
+        <v>$6,157.29</v>
       </c>
     </row>
     <row r="8">
@@ -486,13 +486,13 @@
         <v>Mayo</v>
       </c>
       <c r="B8" t="str">
-        <v>3,351.463</v>
+        <v>3,243.688</v>
       </c>
       <c r="C8" t="str">
-        <v>$12,456.36</v>
+        <v>$12,902.79</v>
       </c>
       <c r="D8" t="str">
-        <v>$5,806.24</v>
+        <v>$6,521.80</v>
       </c>
     </row>
     <row r="9">
@@ -500,13 +500,13 @@
         <v>Junio</v>
       </c>
       <c r="B9" t="str">
-        <v>3,067.326</v>
+        <v>3,568.003</v>
       </c>
       <c r="C9" t="str">
-        <v>$13,882.22</v>
+        <v>$13,163.21</v>
       </c>
       <c r="D9" t="str">
-        <v>$5,822.64</v>
+        <v>$5,666.66</v>
       </c>
     </row>
     <row r="10">
@@ -514,13 +514,13 @@
         <v>Julio</v>
       </c>
       <c r="B10" t="str">
-        <v>3,825.894</v>
+        <v>3,777.758</v>
       </c>
       <c r="C10" t="str">
-        <v>$14,488.80</v>
+        <v>$12,652.38</v>
       </c>
       <c r="D10" t="str">
-        <v>$6,244.71</v>
+        <v>$6,347.35</v>
       </c>
     </row>
     <row r="11">
@@ -528,13 +528,13 @@
         <v>Agosto</v>
       </c>
       <c r="B11" t="str">
-        <v>3,269.638</v>
+        <v>3,533.799</v>
       </c>
       <c r="C11" t="str">
-        <v>$12,153.26</v>
+        <v>$13,091.77</v>
       </c>
       <c r="D11" t="str">
-        <v>$6,151.04</v>
+        <v>$5,236.13</v>
       </c>
     </row>
     <row r="12">
@@ -542,13 +542,13 @@
         <v>Septiembre</v>
       </c>
       <c r="B12" t="str">
-        <v>3,367.017</v>
+        <v>3,054.76</v>
       </c>
       <c r="C12" t="str">
-        <v>$12,163.81</v>
+        <v>$13,617.42</v>
       </c>
       <c r="D12" t="str">
-        <v>$5,772.56</v>
+        <v>$6,743.58</v>
       </c>
     </row>
     <row r="13">
@@ -556,13 +556,13 @@
         <v>Octubre</v>
       </c>
       <c r="B13" t="str">
-        <v>3,067.208</v>
+        <v>3,329.853</v>
       </c>
       <c r="C13" t="str">
-        <v>$12,621.95</v>
+        <v>$13,756.91</v>
       </c>
       <c r="D13" t="str">
-        <v>$6,898.68</v>
+        <v>$6,025.75</v>
       </c>
     </row>
     <row r="14">
@@ -570,13 +570,13 @@
         <v>Noviembre</v>
       </c>
       <c r="B14" t="str">
-        <v>3,687.713</v>
+        <v>3,336.189</v>
       </c>
       <c r="C14" t="str">
-        <v>$13,854.80</v>
+        <v>$13,220.98</v>
       </c>
       <c r="D14" t="str">
-        <v>$6,040.37</v>
+        <v>$5,259.71</v>
       </c>
     </row>
     <row r="15">
@@ -584,13 +584,13 @@
         <v>Diciembre</v>
       </c>
       <c r="B15" t="str">
-        <v>3,747.613</v>
+        <v>3,920.637</v>
       </c>
       <c r="C15" t="str">
-        <v>$12,278.59</v>
+        <v>$14,678.02</v>
       </c>
       <c r="D15" t="str">
-        <v>$5,987.60</v>
+        <v>$6,245.05</v>
       </c>
     </row>
   </sheetData>
@@ -634,13 +634,13 @@
         <v>Promedio</v>
       </c>
       <c r="B4" t="str">
-        <v>3,561.805</v>
+        <v>3,407.057</v>
       </c>
       <c r="C4" t="str">
-        <v>$12,929.53</v>
+        <v>$13,527.61</v>
       </c>
       <c r="D4" t="str">
-        <v>$6,072.96</v>
+        <v>$5,917.20</v>
       </c>
     </row>
     <row r="5">
@@ -648,13 +648,13 @@
         <v>Máximo</v>
       </c>
       <c r="B5" t="str">
-        <v>3,921.754</v>
+        <v>3,920.637</v>
       </c>
       <c r="C5" t="str">
-        <v>$14,488.80</v>
+        <v>$14,921.71</v>
       </c>
       <c r="D5" t="str">
-        <v>$6,898.68</v>
+        <v>$6,743.58</v>
       </c>
     </row>
     <row r="6">
@@ -662,13 +662,13 @@
         <v>Mínimo</v>
       </c>
       <c r="B6" t="str">
-        <v>3,067.208</v>
+        <v>3,054.76</v>
       </c>
       <c r="C6" t="str">
-        <v>$12,072.04</v>
+        <v>$12,195.96</v>
       </c>
       <c r="D6" t="str">
-        <v>$5,613.19</v>
+        <v>$5,009.56</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Checkpoint: Implementar lectura correcta de wallet balance: 1. getWalletSummary: Ahora calcula completedReservesAmount (suma de reservas con status='completed') y reservedPendingAmount (suma de status='suggested' o 'approved') 2. getPartnerSummary: Retorna datos reales de socios (Wascar, Yisvel) con participationPercent y totalDrawn 3. Ambos endpoints retornan datos en lugar de placeholders vacíos 4. Tests unitarios para validar lógica de cálculos 5. Sin tocar Plaid, Sync, Reserve generation, Dismiss
</commit_message>
<xml_diff>
--- a/comparison.xlsx
+++ b/comparison.xlsx
@@ -430,13 +430,13 @@
         <v>Enero</v>
       </c>
       <c r="B4" t="str">
-        <v>3,155.89</v>
+        <v>3,736.896</v>
       </c>
       <c r="C4" t="str">
-        <v>$14,921.71</v>
+        <v>$14,661.67</v>
       </c>
       <c r="D4" t="str">
-        <v>$5,009.56</v>
+        <v>$5,409.41</v>
       </c>
     </row>
     <row r="5">
@@ -444,13 +444,13 @@
         <v>Febrero</v>
       </c>
       <c r="B5" t="str">
-        <v>3,613.509</v>
+        <v>3,087.334</v>
       </c>
       <c r="C5" t="str">
-        <v>$14,837.88</v>
+        <v>$13,885.97</v>
       </c>
       <c r="D5" t="str">
-        <v>$5,531.33</v>
+        <v>$6,439.86</v>
       </c>
     </row>
     <row r="6">
@@ -458,13 +458,13 @@
         <v>Marzo</v>
       </c>
       <c r="B6" t="str">
-        <v>3,061.74</v>
+        <v>3,109.569</v>
       </c>
       <c r="C6" t="str">
-        <v>$12,195.96</v>
+        <v>$13,734.01</v>
       </c>
       <c r="D6" t="str">
-        <v>$6,262.18</v>
+        <v>$6,552.34</v>
       </c>
     </row>
     <row r="7">
@@ -472,13 +472,13 @@
         <v>Abril</v>
       </c>
       <c r="B7" t="str">
-        <v>3,288.855</v>
+        <v>3,712.87</v>
       </c>
       <c r="C7" t="str">
-        <v>$13,292.28</v>
+        <v>$14,132.85</v>
       </c>
       <c r="D7" t="str">
-        <v>$6,157.29</v>
+        <v>$5,255.41</v>
       </c>
     </row>
     <row r="8">
@@ -486,13 +486,13 @@
         <v>Mayo</v>
       </c>
       <c r="B8" t="str">
-        <v>3,243.688</v>
+        <v>3,899.506</v>
       </c>
       <c r="C8" t="str">
-        <v>$12,902.79</v>
+        <v>$13,158.17</v>
       </c>
       <c r="D8" t="str">
-        <v>$6,521.80</v>
+        <v>$5,086.02</v>
       </c>
     </row>
     <row r="9">
@@ -500,13 +500,13 @@
         <v>Junio</v>
       </c>
       <c r="B9" t="str">
-        <v>3,568.003</v>
+        <v>3,456.187</v>
       </c>
       <c r="C9" t="str">
-        <v>$13,163.21</v>
+        <v>$14,704.60</v>
       </c>
       <c r="D9" t="str">
-        <v>$5,666.66</v>
+        <v>$5,224.41</v>
       </c>
     </row>
     <row r="10">
@@ -514,13 +514,13 @@
         <v>Julio</v>
       </c>
       <c r="B10" t="str">
-        <v>3,777.758</v>
+        <v>3,350.126</v>
       </c>
       <c r="C10" t="str">
-        <v>$12,652.38</v>
+        <v>$14,960.06</v>
       </c>
       <c r="D10" t="str">
-        <v>$6,347.35</v>
+        <v>$6,662.19</v>
       </c>
     </row>
     <row r="11">
@@ -528,13 +528,13 @@
         <v>Agosto</v>
       </c>
       <c r="B11" t="str">
-        <v>3,533.799</v>
+        <v>3,772.608</v>
       </c>
       <c r="C11" t="str">
-        <v>$13,091.77</v>
+        <v>$14,593.97</v>
       </c>
       <c r="D11" t="str">
-        <v>$5,236.13</v>
+        <v>$5,740.76</v>
       </c>
     </row>
     <row r="12">
@@ -542,13 +542,13 @@
         <v>Septiembre</v>
       </c>
       <c r="B12" t="str">
-        <v>3,054.76</v>
+        <v>3,603.883</v>
       </c>
       <c r="C12" t="str">
-        <v>$13,617.42</v>
+        <v>$12,101.28</v>
       </c>
       <c r="D12" t="str">
-        <v>$6,743.58</v>
+        <v>$6,012.82</v>
       </c>
     </row>
     <row r="13">
@@ -556,13 +556,13 @@
         <v>Octubre</v>
       </c>
       <c r="B13" t="str">
-        <v>3,329.853</v>
+        <v>3,311.749</v>
       </c>
       <c r="C13" t="str">
-        <v>$13,756.91</v>
+        <v>$12,983.22</v>
       </c>
       <c r="D13" t="str">
-        <v>$6,025.75</v>
+        <v>$5,866.90</v>
       </c>
     </row>
     <row r="14">
@@ -570,13 +570,13 @@
         <v>Noviembre</v>
       </c>
       <c r="B14" t="str">
-        <v>3,336.189</v>
+        <v>3,823.75</v>
       </c>
       <c r="C14" t="str">
-        <v>$13,220.98</v>
+        <v>$13,784.22</v>
       </c>
       <c r="D14" t="str">
-        <v>$5,259.71</v>
+        <v>$5,966.48</v>
       </c>
     </row>
     <row r="15">
@@ -584,13 +584,13 @@
         <v>Diciembre</v>
       </c>
       <c r="B15" t="str">
-        <v>3,920.637</v>
+        <v>3,643.758</v>
       </c>
       <c r="C15" t="str">
-        <v>$14,678.02</v>
+        <v>$12,395.82</v>
       </c>
       <c r="D15" t="str">
-        <v>$6,245.05</v>
+        <v>$5,229.87</v>
       </c>
     </row>
   </sheetData>
@@ -634,13 +634,13 @@
         <v>Promedio</v>
       </c>
       <c r="B4" t="str">
-        <v>3,407.057</v>
+        <v>3,542.353</v>
       </c>
       <c r="C4" t="str">
-        <v>$13,527.61</v>
+        <v>$13,757.99</v>
       </c>
       <c r="D4" t="str">
-        <v>$5,917.20</v>
+        <v>$5,787.21</v>
       </c>
     </row>
     <row r="5">
@@ -648,13 +648,13 @@
         <v>Máximo</v>
       </c>
       <c r="B5" t="str">
-        <v>3,920.637</v>
+        <v>3,899.506</v>
       </c>
       <c r="C5" t="str">
-        <v>$14,921.71</v>
+        <v>$14,960.06</v>
       </c>
       <c r="D5" t="str">
-        <v>$6,743.58</v>
+        <v>$6,662.19</v>
       </c>
     </row>
     <row r="6">
@@ -662,13 +662,13 @@
         <v>Mínimo</v>
       </c>
       <c r="B6" t="str">
-        <v>3,054.76</v>
+        <v>3,087.334</v>
       </c>
       <c r="C6" t="str">
-        <v>$12,195.96</v>
+        <v>$12,101.28</v>
       </c>
       <c r="D6" t="str">
-        <v>$5,009.56</v>
+        <v>$5,086.02</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: compact advisor + data-quality visibility in dispatch board
- Add blocked recommendation filter option
- Add data-quality filter (all/reliable/missing)
- Add Needs Backfill badge to DispatchLoadCard and DispatchTableView
- Enhance compact advisor display with financial metrics
- Verify highlighted-load UX (useHighlightedLoad + LoadHighlightWrapper)
- All stability rules maintained, zero new errors
</commit_message>
<xml_diff>
--- a/comparison.xlsx
+++ b/comparison.xlsx
@@ -430,13 +430,13 @@
         <v>Enero</v>
       </c>
       <c r="B4" t="str">
-        <v>3,204.736</v>
+        <v>3,500.252</v>
       </c>
       <c r="C4" t="str">
-        <v>$14,198.91</v>
+        <v>$14,317.37</v>
       </c>
       <c r="D4" t="str">
-        <v>$5,905.52</v>
+        <v>$5,516.74</v>
       </c>
     </row>
     <row r="5">
@@ -444,13 +444,13 @@
         <v>Febrero</v>
       </c>
       <c r="B5" t="str">
-        <v>3,936.003</v>
+        <v>3,298.652</v>
       </c>
       <c r="C5" t="str">
-        <v>$13,446.48</v>
+        <v>$12,714.56</v>
       </c>
       <c r="D5" t="str">
-        <v>$5,680.72</v>
+        <v>$5,160.95</v>
       </c>
     </row>
     <row r="6">
@@ -458,13 +458,13 @@
         <v>Marzo</v>
       </c>
       <c r="B6" t="str">
-        <v>3,997.963</v>
+        <v>3,989.764</v>
       </c>
       <c r="C6" t="str">
-        <v>$13,209.33</v>
+        <v>$12,084.13</v>
       </c>
       <c r="D6" t="str">
-        <v>$6,966.18</v>
+        <v>$6,093.76</v>
       </c>
     </row>
     <row r="7">
@@ -472,13 +472,13 @@
         <v>Abril</v>
       </c>
       <c r="B7" t="str">
-        <v>3,962.365</v>
+        <v>3,476.868</v>
       </c>
       <c r="C7" t="str">
-        <v>$13,259.79</v>
+        <v>$12,762.02</v>
       </c>
       <c r="D7" t="str">
-        <v>$6,632.13</v>
+        <v>$6,290.90</v>
       </c>
     </row>
     <row r="8">
@@ -486,13 +486,13 @@
         <v>Mayo</v>
       </c>
       <c r="B8" t="str">
-        <v>3,672.273</v>
+        <v>3,127.437</v>
       </c>
       <c r="C8" t="str">
-        <v>$13,128.76</v>
+        <v>$12,213.84</v>
       </c>
       <c r="D8" t="str">
-        <v>$5,700.39</v>
+        <v>$6,732.10</v>
       </c>
     </row>
     <row r="9">
@@ -500,13 +500,13 @@
         <v>Junio</v>
       </c>
       <c r="B9" t="str">
-        <v>3,129.573</v>
+        <v>3,258.744</v>
       </c>
       <c r="C9" t="str">
-        <v>$13,301.86</v>
+        <v>$13,238.62</v>
       </c>
       <c r="D9" t="str">
-        <v>$5,219.76</v>
+        <v>$6,620.20</v>
       </c>
     </row>
     <row r="10">
@@ -514,13 +514,13 @@
         <v>Julio</v>
       </c>
       <c r="B10" t="str">
-        <v>3,706.874</v>
+        <v>3,687.167</v>
       </c>
       <c r="C10" t="str">
-        <v>$12,884.43</v>
+        <v>$13,823.22</v>
       </c>
       <c r="D10" t="str">
-        <v>$5,510.47</v>
+        <v>$5,451.21</v>
       </c>
     </row>
     <row r="11">
@@ -528,13 +528,13 @@
         <v>Agosto</v>
       </c>
       <c r="B11" t="str">
-        <v>3,587.19</v>
+        <v>3,791.328</v>
       </c>
       <c r="C11" t="str">
-        <v>$14,109.76</v>
+        <v>$14,837.06</v>
       </c>
       <c r="D11" t="str">
-        <v>$5,711.99</v>
+        <v>$6,908.94</v>
       </c>
     </row>
     <row r="12">
@@ -542,13 +542,13 @@
         <v>Septiembre</v>
       </c>
       <c r="B12" t="str">
-        <v>3,681.297</v>
+        <v>3,638.112</v>
       </c>
       <c r="C12" t="str">
-        <v>$14,135.28</v>
+        <v>$12,347.96</v>
       </c>
       <c r="D12" t="str">
-        <v>$6,014.62</v>
+        <v>$5,899.77</v>
       </c>
     </row>
     <row r="13">
@@ -556,13 +556,13 @@
         <v>Octubre</v>
       </c>
       <c r="B13" t="str">
-        <v>3,440.348</v>
+        <v>3,489.4</v>
       </c>
       <c r="C13" t="str">
-        <v>$13,297.82</v>
+        <v>$13,536.37</v>
       </c>
       <c r="D13" t="str">
-        <v>$5,929.51</v>
+        <v>$6,791.83</v>
       </c>
     </row>
     <row r="14">
@@ -570,13 +570,13 @@
         <v>Noviembre</v>
       </c>
       <c r="B14" t="str">
-        <v>3,868.074</v>
+        <v>3,652.213</v>
       </c>
       <c r="C14" t="str">
-        <v>$14,091.57</v>
+        <v>$13,144.76</v>
       </c>
       <c r="D14" t="str">
-        <v>$5,234.83</v>
+        <v>$6,184.38</v>
       </c>
     </row>
     <row r="15">
@@ -584,13 +584,13 @@
         <v>Diciembre</v>
       </c>
       <c r="B15" t="str">
-        <v>3,019.66</v>
+        <v>3,879.147</v>
       </c>
       <c r="C15" t="str">
-        <v>$13,287.61</v>
+        <v>$13,096.44</v>
       </c>
       <c r="D15" t="str">
-        <v>$6,184.09</v>
+        <v>$5,655.29</v>
       </c>
     </row>
   </sheetData>
@@ -634,13 +634,13 @@
         <v>Promedio</v>
       </c>
       <c r="B4" t="str">
-        <v>3,600.53</v>
+        <v>3,565.757</v>
       </c>
       <c r="C4" t="str">
-        <v>$13,529.30</v>
+        <v>$13,176.36</v>
       </c>
       <c r="D4" t="str">
-        <v>$5,890.85</v>
+        <v>$6,108.84</v>
       </c>
     </row>
     <row r="5">
@@ -648,13 +648,13 @@
         <v>Máximo</v>
       </c>
       <c r="B5" t="str">
-        <v>3,997.963</v>
+        <v>3,989.764</v>
       </c>
       <c r="C5" t="str">
-        <v>$14,198.91</v>
+        <v>$14,837.06</v>
       </c>
       <c r="D5" t="str">
-        <v>$6,966.18</v>
+        <v>$6,908.94</v>
       </c>
     </row>
     <row r="6">
@@ -662,13 +662,13 @@
         <v>Mínimo</v>
       </c>
       <c r="B6" t="str">
-        <v>3,019.66</v>
+        <v>3,127.437</v>
       </c>
       <c r="C6" t="str">
-        <v>$12,884.43</v>
+        <v>$12,084.13</v>
       </c>
       <c r="D6" t="str">
-        <v>$5,219.76</v>
+        <v>$5,160.95</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Checkpoint: Fixed useAuth import path in routeGuards.tsx from @/_core/hooks/useAuth to @/contexts/AuthContext to ensure consistent auth state access. Build successful with no TypeScript errors.
</commit_message>
<xml_diff>
--- a/comparison.xlsx
+++ b/comparison.xlsx
@@ -430,13 +430,13 @@
         <v>Enero</v>
       </c>
       <c r="B4" t="str">
-        <v>3,500.252</v>
+        <v>3,615.749</v>
       </c>
       <c r="C4" t="str">
-        <v>$14,317.37</v>
+        <v>$14,838.75</v>
       </c>
       <c r="D4" t="str">
-        <v>$5,516.74</v>
+        <v>$6,499.15</v>
       </c>
     </row>
     <row r="5">
@@ -444,13 +444,13 @@
         <v>Febrero</v>
       </c>
       <c r="B5" t="str">
-        <v>3,298.652</v>
+        <v>3,410.082</v>
       </c>
       <c r="C5" t="str">
-        <v>$12,714.56</v>
+        <v>$13,267.38</v>
       </c>
       <c r="D5" t="str">
-        <v>$5,160.95</v>
+        <v>$6,954.58</v>
       </c>
     </row>
     <row r="6">
@@ -458,13 +458,13 @@
         <v>Marzo</v>
       </c>
       <c r="B6" t="str">
-        <v>3,989.764</v>
+        <v>3,939.392</v>
       </c>
       <c r="C6" t="str">
-        <v>$12,084.13</v>
+        <v>$12,858.42</v>
       </c>
       <c r="D6" t="str">
-        <v>$6,093.76</v>
+        <v>$5,353.78</v>
       </c>
     </row>
     <row r="7">
@@ -472,13 +472,13 @@
         <v>Abril</v>
       </c>
       <c r="B7" t="str">
-        <v>3,476.868</v>
+        <v>3,372.002</v>
       </c>
       <c r="C7" t="str">
-        <v>$12,762.02</v>
+        <v>$14,388.04</v>
       </c>
       <c r="D7" t="str">
-        <v>$6,290.90</v>
+        <v>$6,188.52</v>
       </c>
     </row>
     <row r="8">
@@ -486,13 +486,13 @@
         <v>Mayo</v>
       </c>
       <c r="B8" t="str">
-        <v>3,127.437</v>
+        <v>3,495.814</v>
       </c>
       <c r="C8" t="str">
-        <v>$12,213.84</v>
+        <v>$13,671.41</v>
       </c>
       <c r="D8" t="str">
-        <v>$6,732.10</v>
+        <v>$5,590.07</v>
       </c>
     </row>
     <row r="9">
@@ -500,13 +500,13 @@
         <v>Junio</v>
       </c>
       <c r="B9" t="str">
-        <v>3,258.744</v>
+        <v>3,907.817</v>
       </c>
       <c r="C9" t="str">
-        <v>$13,238.62</v>
+        <v>$14,411.84</v>
       </c>
       <c r="D9" t="str">
-        <v>$6,620.20</v>
+        <v>$6,977.37</v>
       </c>
     </row>
     <row r="10">
@@ -514,13 +514,13 @@
         <v>Julio</v>
       </c>
       <c r="B10" t="str">
-        <v>3,687.167</v>
+        <v>3,990.975</v>
       </c>
       <c r="C10" t="str">
-        <v>$13,823.22</v>
+        <v>$14,544.09</v>
       </c>
       <c r="D10" t="str">
-        <v>$5,451.21</v>
+        <v>$5,763.69</v>
       </c>
     </row>
     <row r="11">
@@ -528,13 +528,13 @@
         <v>Agosto</v>
       </c>
       <c r="B11" t="str">
-        <v>3,791.328</v>
+        <v>3,362.765</v>
       </c>
       <c r="C11" t="str">
-        <v>$14,837.06</v>
+        <v>$13,049.94</v>
       </c>
       <c r="D11" t="str">
-        <v>$6,908.94</v>
+        <v>$6,420.19</v>
       </c>
     </row>
     <row r="12">
@@ -542,13 +542,13 @@
         <v>Septiembre</v>
       </c>
       <c r="B12" t="str">
-        <v>3,638.112</v>
+        <v>3,548.289</v>
       </c>
       <c r="C12" t="str">
-        <v>$12,347.96</v>
+        <v>$13,299.79</v>
       </c>
       <c r="D12" t="str">
-        <v>$5,899.77</v>
+        <v>$5,488.38</v>
       </c>
     </row>
     <row r="13">
@@ -556,13 +556,13 @@
         <v>Octubre</v>
       </c>
       <c r="B13" t="str">
-        <v>3,489.4</v>
+        <v>3,717.707</v>
       </c>
       <c r="C13" t="str">
-        <v>$13,536.37</v>
+        <v>$13,166.07</v>
       </c>
       <c r="D13" t="str">
-        <v>$6,791.83</v>
+        <v>$5,183.74</v>
       </c>
     </row>
     <row r="14">
@@ -570,13 +570,13 @@
         <v>Noviembre</v>
       </c>
       <c r="B14" t="str">
-        <v>3,652.213</v>
+        <v>3,499.61</v>
       </c>
       <c r="C14" t="str">
-        <v>$13,144.76</v>
+        <v>$13,699.72</v>
       </c>
       <c r="D14" t="str">
-        <v>$6,184.38</v>
+        <v>$5,527.57</v>
       </c>
     </row>
     <row r="15">
@@ -584,13 +584,13 @@
         <v>Diciembre</v>
       </c>
       <c r="B15" t="str">
-        <v>3,879.147</v>
+        <v>3,972.957</v>
       </c>
       <c r="C15" t="str">
-        <v>$13,096.44</v>
+        <v>$14,560.03</v>
       </c>
       <c r="D15" t="str">
-        <v>$5,655.29</v>
+        <v>$6,192.30</v>
       </c>
     </row>
   </sheetData>
@@ -634,13 +634,13 @@
         <v>Promedio</v>
       </c>
       <c r="B4" t="str">
-        <v>3,565.757</v>
+        <v>3,652.763</v>
       </c>
       <c r="C4" t="str">
-        <v>$13,176.36</v>
+        <v>$13,812.96</v>
       </c>
       <c r="D4" t="str">
-        <v>$6,108.84</v>
+        <v>$6,011.61</v>
       </c>
     </row>
     <row r="5">
@@ -648,13 +648,13 @@
         <v>Máximo</v>
       </c>
       <c r="B5" t="str">
-        <v>3,989.764</v>
+        <v>3,990.975</v>
       </c>
       <c r="C5" t="str">
-        <v>$14,837.06</v>
+        <v>$14,838.75</v>
       </c>
       <c r="D5" t="str">
-        <v>$6,908.94</v>
+        <v>$6,977.37</v>
       </c>
     </row>
     <row r="6">
@@ -662,13 +662,13 @@
         <v>Mínimo</v>
       </c>
       <c r="B6" t="str">
-        <v>3,127.437</v>
+        <v>3,362.765</v>
       </c>
       <c r="C6" t="str">
-        <v>$12,084.13</v>
+        <v>$12,858.42</v>
       </c>
       <c r="D6" t="str">
-        <v>$5,160.95</v>
+        <v>$5,183.74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>